<commit_message>
RMES as BDF's 8 fields, live-tested in dev (29 Oct)
- RMES: one read-only sheet of the 8 fields BDF named, filled from the CIQ,
  on an RMES tab for Safety and Regulatory only; criteria, limits, AI text
  and findings removed; the department decision moves to the Questionnaire tab.
- Record time: Kissflow form list rows carry no _created_at (proven live), so
  the RMES record time comes from its rmes.saved creation row; the tab names a
  record without a known time.
- Live suites: step 5 / S4 report "blocked" while I-2's Approve is refused
  (no member in Integration service; the reviews are I-2's last step since
  25 Oct), guarded so it hides no other failure; the fake I-2 follows that
  order; new offline S4 rehearsal; read-only S-RMES-PROBE (live/rmes.live.ts).
- Dev: app ciq-app-ui-cfd65e5766, portal ciq-portal-ui-233cc982e5 (Live);
  Bundle.gs 93ce7ec1; MORNING-2026-10-29.md, BDF reply draft.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kissflow-build/CIQ-UAT-test-cases.xlsx
+++ b/kissflow-build/CIQ-UAT-test-cases.xlsx
@@ -957,7 +957,7 @@
           <t>- RMM opens on the Dashboard. The menu is headed “Raw Material Manager (RMM)” and shows only Dashboard, My reviews, Cases and Suppliers. If no case exists yet, the Dashboard shows only “Start your first CIQ case” with “New case” and “Suppliers (n)”.
 - The bottom of the menu shows “Updated hh:mm”, Reload and the night-mode switch. The menu collapses to icons and expands again; Reload updates the time.
 - Each reviewer opens on “My reviews” with the department name above the title (e.g. “Product Safety”). The menu shows only My reviews and Cases. Without a task the page shows “No review tasks yet”.
-- Only the Safety and Regulatory page subtitles mention the internal RMES evaluation and its decision.
+- Only the Safety and Regulatory page subtitles mention their internal decision and the RMES tab (“The RMES tab shows the material's evaluation sheet, filled automatically from the CIQ.”).
 - The Business administrator opens on Rules. The menu shows Rules, Questionnaire, Section owners and Suppliers; there is no Dashboard, My reviews or New case.</t>
         </is>
       </c>
@@ -1730,7 +1730,7 @@
 - Step 4: “My review”: “Your review of the whole CIQ is open”.
 - Step 5: each named reviewer finds the case under To review with “In review”.
 - Step 6: the department that is not concerned has no row. The case page is read-only, with no “Open my review” button.
-- Step 7: the RMES tab shows “Record created &lt;date&gt; for &lt;case ID&gt;”.
+- Step 7: the RMES tab shows “RMES · &lt;case ID&gt; · internal: never visible to the supplier · filled automatically from the CIQ” and “Record created &lt;date, time&gt;”, with the case's 8 fields (TC-26).
 - Step 8: the Dashboard shows “Origin without rules: Waste / side stream”, and the RMM review shows “Flagged for you: origin without rules”. It does not block any completion.</t>
         </is>
       </c>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>REQ-RMES-011, REQ-CTL-003</t>
+          <t>REQ-CTL-003</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>REQ-PROC-007, REQ-PROC-016, REQ-PROC-031, REQ-PROC-011, REQ-CFG-008, REQ-CFG-009, REQ-RMES-012</t>
+          <t>REQ-PROC-007, REQ-PROC-016, REQ-PROC-031, REQ-PROC-011, REQ-CFG-008, REQ-CFG-009</t>
         </is>
       </c>
       <c r="I18" s="9" t="inlineStr">
@@ -1976,12 +1976,12 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>- The window “Ask the supplier” shows the exact answer as the reference. It says “The supplier sees the reference, the question, the justification and the due date. Internal notes, RMES results and findings stay internal.” and “E-mail to &lt;case contacts&gt; (no internal content).”
+          <t>- The window “Ask the supplier” shows the exact answer as the reference. It says “The supplier sees the reference, the question, the justification and the due date. Internal notes, the RMES and the Safety and Regulatory decisions stay internal.” and “E-mail to &lt;case contacts&gt; (no internal content).”
 - Step 3: “Write the question the supplier should answer.” and “Say why Beiersdorf needs this.” Nothing is sent.
 - Step 4: “Pick today or a later date.” Nothing is sent.
 - Step 5: “My open points (1)” shows the point with the reference and question, “Due &lt;date&gt; · Round 1 · Raised by you · Responsible &lt;name&gt; · Why: &lt;justification&gt;” and “With the supplier, waiting for an answer.” “My Safety review” shows “Waiting for supplier”; the bottom bar shows “1 item blocks your completion”.
 - Step 6: the case is under “Waiting for supplier”.
-- Step 7: the request is under “Needs your action”; “Questions for you” shows “1 waiting for your answer” with the reference, question, justification, due date and the asker. The reference jumps to the exact answer. No internal note, RMES result or finding is visible.</t>
+- Step 7: the request is under “Needs your action”; “Questions for you” shows “1 waiting for your answer” with the reference, question, justification, due date and the asker. The reference jumps to the exact answer. No internal note, RMES content or decision is visible.</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>REQ-PROC-033, REQ-PROC-034, REQ-PROC-035, REQ-ADR-001, REQ-RMES-011, REQ-CTL-010</t>
+          <t>REQ-PROC-033, REQ-PROC-034, REQ-PROC-035, REQ-ADR-001, REQ-CTL-010</t>
         </is>
       </c>
       <c r="I25" s="9" t="inlineStr">
@@ -2415,7 +2415,7 @@
       <c r="L26" s="10" t="inlineStr"/>
       <c r="M26" s="11" t="inlineStr"/>
     </row>
-    <row r="27" ht="187.5" customHeight="1">
+    <row r="27" ht="512.5" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>TC-26</t>
@@ -2423,50 +2423,54 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>RMES evaluation</t>
+          <t>RMES</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Product Safety reviewer (repeat as Regulatory Affairs); RMM and Supplier contact (to check)</t>
+          <t>Product Safety reviewer (repeat as Regulatory Affairs); RMM, Quality Management reviewer and Supplier contact (to check)</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Record RMES criterion results with source, limits and required comments</t>
+          <t>RMES shows the 8 fields filled automatically, with their CIQ sources (Safety and Regulatory)</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>A case in review with Safety and Regulatory tasks. K2.2 holds heavy-metal values.</t>
+          <t>A case in review with Safety and Regulatory tasks. In K2.1 the supplier entered at least three components: two of the same origin (e.g. Vegetable (bio mass)) and one of another origin, one of them without CAS and EC number. K2.3 holds the specification of each origin used (for Vegetable or Animal: Part(s) used and Country of origin). In General the supplier answered “Manufacturer (name and address)”.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>1. In the review workspace, open the tab “RMES · Safety”. Read the header and Parts A to D.
-2. On a criterion, click its source link.
-3. On a criterion with a limit, compare the value with the BDF limit.
-4. Choose “Negative”, leave the comment empty and click “Save result”.
-5. Add the comment and save. Record “Available” or “Plausible” on another criterion without a comment.
-6. Click “Change result” on a saved criterion and save it again.
+          <t>1. As the Safety reviewer, open the case from My reviews and click the tab “RMES” next to “Questionnaire”.
+2. Read the header: Raw material / tradename, Supplier and Manufacturer.
+3. Click the source line under Manufacturer.
+4. Go back to the RMES tab and read the Composition table and the line below it.
+5. In the Free text column, click the source line of one text.
+6. Look for anything on the RMES tab that you can type, choose or record.
 7. As the Regulatory reviewer, open the same case's RMES tab.
-8. As RMM, open the case &gt; Overview. As the supplier, open the request.</t>
+8. As RMM and as the Quality Management reviewer, open the case's review workspace. As RMM, also open the case page &gt; Overview.
+9. As the supplier, open the request and its questions.</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>- The header reads “RMES — Safety evaluation” and “Record created &lt;date&gt; for &lt;case ID&gt; · internal, never visible to the supplier”, with “Criteria with a result x of y”.
-- Step 2: the link opens the answer or document the criterion is based on.
-- Step 3: the limit box shows the value, “BDF limit ≤ …”, “Within limit” or “Above limit”, and the limit set used.
-- Step 4: “A comment is required for a negative, implausible or not-applicable result.” Nothing is saved.
-- Steps 5–6: each result shows with comment, name and time; the progress counts up.
-- Step 7: the Regulatory reviewer sees “Safety criteria — read only” and cannot change them.
-- Step 8: RMM sees “RMES progress” with Safety and Regulatory shown separately. Nothing of the RMES appears in the Supplier Portal.</t>
+          <t>- Step 1: the tab is named “RMES” (no count). It shows “Raw Material Evaluation Sheet” with “RMES · &lt;case ID&gt; · internal: never visible to the supplier · filled automatically from the CIQ” and “Record created &lt;date, time&gt;”.
+- Step 2: exactly three header fields. Raw material / tradename shows the trade name, Supplier the supplier's name, and Manufacturer the supplier's answer to “Manufacturer (name and address)”, never the supplier's name in its place. Each shows its CIQ source, e.g. “General · FLD-GEN-004 Manufacturer (name and address)”, and “as of &lt;date, time&gt;”. An unanswered field reads “Not answered yet”; an answer the supplier could not provide reads “Cannot provide: &lt;justification&gt;”.
+- Step 3: the Questionnaire tab opens at General.
+- Step 4: one row per K2.1 component, in the same order, with the columns #, INCI, %, CAS #, EC #, Source of origin and Free text. Each column names its CIQ field (FLD-2.1-001, FLD-2.1-007, FLD-2.1-002, FLD-2.1-003, FLD-2.3-01). % shows the CIQ range, e.g. “90–99 %”, or one value when minimum and maximum are equal. A blank CAS # or EC # shows “—”; EC # may hold a REACH registration number. Source of origin shows the component's origin. Free text shows that origin's specification from K2.3 with its field ID, e.g. “FLD-2.3-11 Fossil specification (e.g. oil, wax, gas)”; for Vegetable and Animal “FLD-2.1-101 Part(s) used” and “FLD-2.3-10 Country of origin”. The rows of the same origin, and a Vegetable row with an Animal row (the CIQ asks Part(s) used and Country of origin once for both), show the same text, marked “*”, and the line below says “The CIQ asks the free text once per origin type, not per component, and asks vegetable and animal together: components of the same origin, or of vegetable and animal origin, show the same text.”
+- Step 5: the Questionnaire tab opens at K2.3.
+- Step 6: nothing on the RMES tab can be edited. There are no criteria, limit checks, suggestions, findings or decision, and no Process ID / RMT ID / IRMA ID or Declaration.
+- Step 7: Regulatory sees the same sheet with the same values.
+- Step 8: RMM and Quality Management have no RMES tab, and the case page shows no RMES card.
+- Step 9: nothing of the RMES is visible to the supplier: not the sheet, its labels or the word “RMES”.
+- If the tab shows “Kissflow did not let your role read this case's questionnaire, so the RMES can't be filled.”, the reviewer's role cannot read the case: record Blocked and name the role.</t>
         </is>
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>REQ-PROC-021, REQ-PROC-022, REQ-RMES-003, REQ-RMES-005, REQ-RMES-006, REQ-RMES-007, REQ-RMES-008, REQ-RMES-015, REQ-RMES-018</t>
+          <t>REQ-PROC-021, REQ-PROC-022, REQ-CFG-004, REQ-RMES-015</t>
         </is>
       </c>
       <c r="I27" s="9" t="inlineStr">
@@ -2487,45 +2491,42 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>RMES evaluation</t>
+          <t>RMES</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Product Safety reviewer; Supplier contact (to check)</t>
+          <t>Supplier contact; Product Safety reviewer (to check)</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Add an internal finding and ask the supplier about it</t>
+          <t>RMES follows a supplier change in Part 2; unchanged after the final release</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>A case in review with a Safety task and its RMES record.</t>
+          <t>TC-26 done. The case is in review and the final release has not been requested yet.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>1. In “RMES · Safety”, click “Add finding” on a criterion. Enter the finding and click “Add finding”.
-2. In the Safety decision card, choose “Approved”.
-3. On the finding, click “Ask supplier”. Write a question for the supplier and click “Send to supplier”.
-4. As the supplier, open the new question.
-5. As the supplier, answer it. As the Safety reviewer, accept the answer and click “Close finding”.</t>
+          <t>1. As the Safety reviewer, open the case's RMES tab and note the values.
+2. As the supplier, open the request. In General, change “Manufacturer (name and address)”. In K2.1, change one component's concentration and add a component of an origin already used. In K2.3, change the specification of one origin used.
+3. As the Safety reviewer, click Reload and open the RMES tab again.
+4. Complete the case: every review completes and the supplier gives the final release (TC-31, TC-32).
+5. As the Safety reviewer, open the completed case from My reviews &gt; Completed and its RMES tab.</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>- Step 1: the finding shows as Open on the criterion and under “Findings”: “Internal. An open finding prevents your approval and your completion.” The bottom bar lists it as a blocker.
-- Step 2: “Not possible yet”: “1 finding is open: close it or reject.”
-- Step 3: the window “Ask the supplier about a finding” uses the criterion's source as reference, marks the finding “Internal finding, not sent” and says the internal finding text is not included. After sending, the finding shows that a question was sent to the supplier; the point is under My open points.
-- Step 4: the supplier sees only the written question and its reference, never the finding text.
-- Step 5: the finding shows Closed and no longer blocks.</t>
+          <t>- Step 3: the sheet shows the new values without anyone copying them: the new manufacturer with a new “as of” time, the new range, the new component in its K2.1 position (marked “*” with the other rows of its origin), and the new specification in every row of that origin. The record line and “Record created” are unchanged. Nothing has to be confirmed or saved on the RMES.
+- Step 5: the sheet shows exactly the released values. They cannot change any more, because the released CIQ is frozen.</t>
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>REQ-RMES-009, REQ-RMES-010, REQ-RMES-015, REQ-PROC-029, REQ-PROC-036</t>
+          <t>REQ-PROC-022, REQ-PROC-016, REQ-PROC-021</t>
         </is>
       </c>
       <c r="I28" s="9" t="inlineStr">
@@ -2538,7 +2539,7 @@
       <c r="L28" s="10" t="inlineStr"/>
       <c r="M28" s="11" t="inlineStr"/>
     </row>
-    <row r="29" ht="200" customHeight="1">
+    <row r="29" ht="362.5" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>TC-28</t>
@@ -2546,49 +2547,54 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>RMES evaluation</t>
+          <t>Safety and Regulatory decision</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Product Safety reviewer; Regulatory Affairs reviewer and RMM (to check); Supplier contact (to check)</t>
+          <t>Product Safety reviewer (repeat as Regulatory Affairs); Regulatory Affairs reviewer and RMM (to check); Supplier contact (to check)</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Record the Safety decision and complete the Safety review</t>
+          <t>Safety/Regulatory decision and completing the review</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>All but one Safety criterion have a result. No Safety finding or Safety open point is open.</t>
+          <t>A case in review with a Safety task and its RMES record (TC-26). No Safety open point is open; no Safety decision is recorded yet.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>1. In “RMES · Safety”, open the “Safety decision” card.
-2. Record the last criterion result. Choose “Approved”, add an optional comment and click “Record approval”.
-3. Read the bottom bar. Click “Change decision”, then “Cancel”.
-4. Click “Complete my review”.
-5. As the Regulatory reviewer, open the same case's RMES tab.
-6. As RMM, open the case &gt; Overview.
-7. As the supplier, open the request.</t>
+          <t>1. In the review workspace, read the bottom bar and expand the list of blocking items.
+2. Click “Record the decision” in the bar.
+3. Read the “Safety decision” card. Choose “Approved”, add an optional comment and click “Record approval”.
+4. Read the bottom bar. Click “Change decision”, then “Cancel”.
+5. Open the RMES tab.
+6. Click “Complete my review”.
+7. As the Regulatory reviewer, open the same case's review workspace.
+8. As RMM, open the case &gt; Overview.
+9. As the supplier, open the request.</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>- Step 1: “Record approval” is disabled with “1 criterion has no result yet.”
-- Step 2: the decision shows “Approved” with name and time. The bar shows “Safety decision: Approved” and “Internal: the supplier never sees it.”
-- Step 3: the bar shows “Nothing blocks your review” and “… It is not a raw-material approval.”
-- Step 4: the bar reads “Product Safety review completed” with name, e-mail, time and “not a raw-material approval”. The case moves to My reviews &gt; Completed.
-- Step 5: Regulatory cannot record or change the Safety decision; it records only its own.
-- Step 6: Reviews shows Product Safety as “Completed” with “Decision: Approved”. Confirmations shows the review completion of Safety with name, e-mail and time.
-- Step 7: the supplier sees no decision and gets no message for this completion.</t>
+          <t>- Step 1: “Safety decision: not recorded yet” with “Record the decision” and “Internal: the supplier never sees it.” The bar reads “1 item blocks your completion”, and the list names “The Safety decision (Approved or Rejected) is not recorded yet”; clicking it goes to the decision card.
+- Step 2: the Questionnaire tab opens with the card “Safety decision” at the top of the right column, above the open points: “Internal. Only Product Safety records it; nobody decides for another department. It is not part of the RMES.”
+- Step 3: the card shows “Approved” with the comment, name and time. The bar shows “Safety decision: Approved” and “Internal: the supplier never sees it.”
+- Step 4: the bar shows “Nothing blocks your review” and “… It is not a raw-material approval.”
+- Step 5: the RMES tab shows only the 8 fields, not the decision.
+- Step 6: the bar reads “Product Safety review completed” with name, e-mail, time and “not a raw-material approval”. The case moves to My reviews &gt; Completed.
+- Step 7: Regulatory has only its own “Regulatory decision” card; it cannot record or change the Safety decision.
+- Step 8: Reviews shows Product Safety as “Completed” with “Decision: Approved”. Confirmations shows the review completion of Safety with name, e-mail and time.
+- Step 9: the supplier sees no decision and gets no message for this completion.
+- Before the case's RMES record exists, the card shows “Not possible yet” and “Record approval” is disabled.</t>
         </is>
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>REQ-RMES-003, REQ-RMES-006, REQ-RMES-013, REQ-PROC-015, REQ-PROC-038, REQ-PROC-039</t>
+          <t>REQ-RMES-013, REQ-PROC-015, REQ-PROC-038, REQ-PROC-039</t>
         </is>
       </c>
       <c r="I29" s="9" t="inlineStr">
@@ -2601,7 +2607,7 @@
       <c r="L29" s="10" t="inlineStr"/>
       <c r="M29" s="11" t="inlineStr"/>
     </row>
-    <row r="30" ht="200" customHeight="1">
+    <row r="30" ht="212.5" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>TC-29</t>
@@ -2609,7 +2615,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>RMES evaluation</t>
+          <t>Safety and Regulatory decision</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -2624,12 +2630,12 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>A case in review. Every Safety criterion has a result. RMM has not completed its own review.</t>
+          <t>A case in review. The Safety reviewer has no open point and no decision on it yet. RMM has not completed its own review.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>1. As the Safety reviewer, choose “Rejected” in the Safety decision card and click “Record rejection” without a reason.
+          <t>1. As the Safety reviewer, open the case's review workspace. On the Questionnaire tab, choose “Rejected” in the “Safety decision” card and click “Record rejection” without a reason.
 2. Enter the reason, record it, and complete the Safety review.
 3. As RMM, open the Dashboard, then the case page.
 4. Click “Decide in my review”. In the bottom bar, click “Choose how to go on”.
@@ -2664,7 +2670,7 @@
       <c r="L30" s="10" t="inlineStr"/>
       <c r="M30" s="11" t="inlineStr"/>
     </row>
-    <row r="31" ht="187.5" customHeight="1">
+    <row r="31" ht="225" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>TC-30</t>
@@ -2703,6 +2709,7 @@
       <c r="G31" s="9" t="inlineStr">
         <is>
           <t>- Step 1: “2 items block your completion”; “Complete my review” is disabled.
+- For Regulatory Affairs the list also names its decision until it is recorded (TC-28).
 - Step 2: each item names its point ID, type, reference, status (“with the supplier” or “answered, waiting for a decision”) and the responsible person. Clicking an item jumps to that point.
 - Step 4: before completing, the bar reads “Nothing blocks your review” and “Confirms your department reviewed everything assigned and no query is open. It is not a raw-material approval.” It names the reviews still to complete before the final-release request goes to the supplier. After completing: “Quality Management review completed”, with name, e-mail, time and “not a raw-material approval”.
 - Step 5: the case is under Completed. Overview shows QM as “Completed”; Confirmations shows its review completion.
@@ -2767,7 +2774,7 @@
 - Step 4: the task “Give the final release” shows “Beiersdorf has completed its review”. The card shows “Final release needed”, “Step 3 of 3 · all Beiersdorf reviews complete · questionnaire locked” and “Give the final release”.
 - Step 5: the card “All Beiersdorf reviews are complete. Please give the final release.” lists Sections in your questionnaire, Documents submitted, Completeness confirmed (name · date), Questions closed (x of y) and Due. The heading reads “Your questionnaire (locked)”; each section shows “Locked: Beiersdorf has requested your final release”. There are no inputs, uploads, “Remove” or justification links.
 - Step 6: B sees “&lt;A&gt; can give the final release for your company.”
-- No decision, finding, RMES result or internal note is shown to the supplier.</t>
+- No decision, RMES content or internal note is shown to the supplier.</t>
         </is>
       </c>
       <c r="H32" s="9" t="inlineStr">
@@ -2885,7 +2892,7 @@
           <t>- The phase is “Completed”, with all four steps done.
 - The green banner reads “Completed &lt;time&gt;. The final document was created automatically at the supplier's final release and sent to &lt;owner&gt;.”
 - Confirmations lists the three kinds separately: Completeness confirmation, Review completion per department, and Final release (Supplier badge, name, role, e-mail, time). None is called a raw-material approval.
-- Step 2: “CIQ final document” with the case ID and “Document seal: unchanged”. It contains the released answers by section with the metadata answers, the K2.1 composition, the evidence list with upload dates, every open point round by round, and all confirmations. It shows no RMES decision, finding or internal note, and cannot be changed.
+- Step 2: “CIQ final document” with the case ID and “Document seal: unchanged”. It contains the released answers by section with the metadata answers, the K2.1 composition, the evidence list with upload dates, every open point round by round, and all confirmations. It shows no RMES content, no Safety or Regulatory decision and no internal note, and cannot be changed.
 - Step 3: the case is listed under Completed and is no longer in “My cases”.
 - Step 4: the workspace shows that the case is completed and the CIQ is frozen.
 - Step 5: the supplier sees “Your released questionnaire”; nothing can be changed.
@@ -3288,7 +3295,7 @@
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Supplier X: contact A is named on request R1, contact B only on R2, contact D on no request (open or closed). A, B and C may confirm and release; D can be the contact marked “May not confirm”. Supplier Y: contact C is named on R3. On R1, reviewers wrote internal notes and RMES results, raised a finding and turned it into a question. User E has a portal account without the supplier role.</t>
+          <t>Supplier X: contact A is named on request R1, contact B only on R2, contact D on no request (open or closed). A, B and C may confirm and release; D can be the contact marked “May not confirm”. Supplier Y: contact C is named on R3. On R1, reviewers wrote internal notes, recorded the Safety and Regulatory decisions with a comment and asked the supplier a question. User E has a portal account without the supplier role.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
@@ -3296,7 +3303,7 @@
           <t>1. As A, sign in and note the listed requests (open and Closed).
 2. As B, sign in and check My requests (open and Closed): R1 is not listed.
 3. As C, sign in and do the same.
-4. As A, open R1 and the question that came from the finding. Read the Help page.
+4. As A, open R1 and the question from Beiersdorf. Read the Help page.
 5. Sign in as E.
 6. As the Business administrator, deactivate contact D. Then sign in as D.</t>
         </is>
@@ -3306,7 +3313,7 @@
           <t>- A sees R1 and only other requests on which A is named.
 - B sees R2 but not R1.
 - C sees only R3.
-- On R1 there are no department names, review statuses or decisions, no RMES criteria or results, no findings, no internal notes, no internal reasons (closing, reopening, cancelling) and no rule numbers. The question from the finding appears as “Question from Beiersdorf”, with no sign of the finding.
+- On R1 there are no department names, review statuses or decisions, nothing of the RMES, no internal notes, no internal reasons (closing, reopening, cancelling) and no rule numbers. The question appears as “Question from Beiersdorf”, with its reference, question, justification and due date only.
 - E sees “No access to the supplier portal”, asking to contact Beiersdorf for an invitation.
 - D sees no request (“No requests yet”). A message that the access has ended is not in this version. Removing D's portal account is done in the portal's user management and is outside this test.</t>
         </is>
@@ -3372,7 +3379,7 @@
       </c>
       <c r="H42" s="9" t="inlineStr">
         <is>
-          <t>REQ-ADR-001, REQ-CTL-003, REQ-CTL-006, REQ-CTL-010, REQ-RMES-019</t>
+          <t>REQ-ADR-001, REQ-CTL-003, REQ-CTL-006, REQ-CTL-010</t>
         </is>
       </c>
       <c r="I42" s="9" t="inlineStr">
@@ -3433,7 +3440,7 @@
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>REQ-CTL-003, REQ-CTL-006, REQ-PROC-036, REQ-RMES-018</t>
+          <t>REQ-CTL-003, REQ-CTL-006, REQ-PROC-036</t>
         </is>
       </c>
       <c r="I43" s="9" t="inlineStr">
@@ -3604,6 +3611,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -3781,6 +3789,7 @@
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="15" t="n"/>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
30 Oct: ready for prod: Bundle.gs rebuilt (eff9ac4776345e16), prod steps fixed, workbook TC-05/TC-31
Bundle.gs from HEAD (documents Mandatory/Optional): offline 54/54, finalPdf.test.ts 6/6.
README: "Update the bundle (prod already set up)" (existing Bundle file, new version of the existing deployment).
TEST-GUIDE-PROD step 7 and PROD-MORNING item 9: no installTrigger, no new project; PROD-MORNING A: upload by hand, portal then app.
Workbook: TC-05 step 5 for the phone section bar; TC-31 no longer Blocked.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kissflow-build/CIQ-UAT-test-cases.xlsx
+++ b/kissflow-build/CIQ-UAT-test-cases.xlsx
@@ -1132,7 +1132,7 @@
 2. Collapse and expand the left menu. Click “How the portal works”, then “My requests”.
 3. Click “Start the questionnaire” on the request card. Read the header, the step bar and the completeness bar.
 4. Read the section navigator and open “General information”.
-5. Repeat on a phone-sized screen and open the section selector.</t>
+5. Repeat on a phone and tap the section bar under the header.</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -1141,7 +1141,7 @@
 - Step 2: the menu has “My requests” with the open-task count and “Help”, and at the bottom “Updated &lt;time&gt;”, Reload and the night-mode switch. Help shows “How it works” in three steps, the FAQs and “Your Beiersdorf contacts”.
 - Step 3: the header names your Beiersdorf contact and the due date. The step bar reads Questionnaire · Beiersdorf review · Final release. The completeness bar shows “0 % complete · 0 of N required answers”, “Every answer is saved automatically.”, “Check completeness” and “Confirm completeness”.
 - Step 4: “&lt;N&gt; sections apply to this material”, grouped into General, Chapters and Annexes, each marked Mandatory, Optional or Documents only. K6.2 and A11 are listed (UK market); Turkey REACH is not. In General information, trade name, supplier, DUNS number and contact e-mails are locked (“Pre-filled by Beiersdorf”); manufacturer and production site can be edited.
-- Step 5: a “Section” selector, grouped the same way; no sideways scrolling.</t>
+- Step 5: no left menu; a bar at the bottom shows “My requests”, “Help” and “More”. The section bar under the header shows the open section and “&lt;n&gt; / &lt;N&gt;” and opens “Sections”, grouped the same way. “Check completeness” and “Confirm completeness” sit in a bar at the bottom; no sideways scrolling.</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Do this test last: once published, new cases use the new version, so step 10 sets it back. No draft version is open; at least one case is running. Steps 4–8 need the update with mandatory and optional documents: if “Upload required?” is not offered in step 4, click “Discard draft” and record Blocked.</t>
+          <t>Do this test last: once published, new cases use the new version, so step 10 sets it back. No draft version is open; at least one case is running.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
@@ -2762,19 +2762,6 @@
       <c r="L32" s="10" t="inlineStr"/>
       <c r="M32" s="11" t="inlineStr"/>
     </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
   </sheetData>
   <autoFilter ref="A1:M32"/>
   <dataValidations count="2">
@@ -2813,7 +2800,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2991,7 +2977,6 @@
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="15" t="n"/>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>

</xml_diff>